<commit_message>
LMS-13 API JWT Auth (Login/Refresh/Logout, không có Register)
</commit_message>
<xml_diff>
--- a/import_template_example.xlsx
+++ b/import_template_example.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Danh sách Nhập" sheetId="1" r:id="rId1"/>
+    <sheet name="Danh sách người dùng" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,14 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,16 +418,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nguyễn Văn A</v>
+        <v>Le Van An</v>
       </c>
       <c r="B2" t="str">
-        <v>nguyenvana@edulms.edu</v>
+        <v>an.student@edulms.edu</v>
       </c>
       <c r="C2" t="str">
-        <v>học sinh</v>
+        <v>student</v>
       </c>
       <c r="D2" t="str">
-        <v>HS-1002</v>
+        <v>HS-9001</v>
       </c>
       <c r="E2" t="str">
         <v>10A1</v>
@@ -442,16 +435,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Trần Thị B</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>tranthib@edulms.edu</v>
+        <v>empty.name@edulms.edu</v>
       </c>
       <c r="C3" t="str">
-        <v>học sinh</v>
+        <v>student</v>
       </c>
       <c r="D3" t="str">
-        <v>HS-1003</v>
+        <v>HS-9002</v>
       </c>
       <c r="E3" t="str">
         <v>10A1</v>
@@ -459,41 +452,330 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ngô Văn C</v>
+        <v>Tran Thi Binh</v>
       </c>
       <c r="B4" t="str">
-        <v>ngovanc@edulms.edu</v>
+        <v>binh@edulms.edu</v>
       </c>
       <c r="C4" t="str">
-        <v>giáo viên</v>
+        <v>invalid_role</v>
       </c>
       <c r="D4" t="str">
-        <v>GV-2003</v>
+        <v>HS-9003</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>10A1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Lê Văn D</v>
+        <v>Nguyen Van Cuong</v>
       </c>
       <c r="B5" t="str">
-        <v>levand@edulms.edu</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>student</v>
       </c>
       <c r="D5" t="str">
-        <v>HS-1004</v>
+        <v>HS-9004</v>
       </c>
       <c r="E5" t="str">
         <v>10A1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Pham Van Dung</v>
+      </c>
+      <c r="B6" t="str">
+        <v>dung_email_invalid</v>
+      </c>
+      <c r="C6" t="str">
+        <v>student</v>
+      </c>
+      <c r="D6" t="str">
+        <v>HS-9005</v>
+      </c>
+      <c r="E6" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Hoang Thi Em</v>
+      </c>
+      <c r="B7" t="str">
+        <v>duplicate.sheet@edulms.edu</v>
+      </c>
+      <c r="C7" t="str">
+        <v>student</v>
+      </c>
+      <c r="D7" t="str">
+        <v>HS-9006</v>
+      </c>
+      <c r="E7" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Hoang Van Giang</v>
+      </c>
+      <c r="B8" t="str">
+        <v>duplicate.sheet@edulms.edu</v>
+      </c>
+      <c r="C8" t="str">
+        <v>student</v>
+      </c>
+      <c r="D8" t="str">
+        <v>HS-9007</v>
+      </c>
+      <c r="E8" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Vu Van Hai</v>
+      </c>
+      <c r="B9" t="str">
+        <v>student@edulms.edu</v>
+      </c>
+      <c r="C9" t="str">
+        <v>student</v>
+      </c>
+      <c r="D9" t="str">
+        <v>HS-9008</v>
+      </c>
+      <c r="E9" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Bui Thi Hoa</v>
+      </c>
+      <c r="B10" t="str">
+        <v>hoa@edulms.edu</v>
+      </c>
+      <c r="C10" t="str">
+        <v>student</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Ngo Van Hung</v>
+      </c>
+      <c r="B11" t="str">
+        <v>hung@edulms.edu</v>
+      </c>
+      <c r="C11" t="str">
+        <v>student</v>
+      </c>
+      <c r="D11" t="str">
+        <v>HS-9009</v>
+      </c>
+      <c r="E11" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Do Van Khanh</v>
+      </c>
+      <c r="B12" t="str">
+        <v>khanh@edulms.edu</v>
+      </c>
+      <c r="C12" t="str">
+        <v>student</v>
+      </c>
+      <c r="D12" t="str">
+        <v>HS-9009</v>
+      </c>
+      <c r="E12" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Dinh Van Lam</v>
+      </c>
+      <c r="B13" t="str">
+        <v>lam@edulms.edu</v>
+      </c>
+      <c r="C13" t="str">
+        <v>student</v>
+      </c>
+      <c r="D13" t="str">
+        <v>HS-1001</v>
+      </c>
+      <c r="E13" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Phan Thi Mai</v>
+      </c>
+      <c r="B14" t="str">
+        <v>mai@edulms.edu</v>
+      </c>
+      <c r="C14" t="str">
+        <v>student</v>
+      </c>
+      <c r="D14" t="str">
+        <v>HS-9010</v>
+      </c>
+      <c r="E14" t="str">
+        <v>10A2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Truong Van Nam</v>
+      </c>
+      <c r="B15" t="str">
+        <v>nam.teacher@edulms.edu</v>
+      </c>
+      <c r="C15" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="D15" t="str">
+        <v>GV-9001</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Vo Van Oanh</v>
+      </c>
+      <c r="B16" t="str">
+        <v>oanh@edulms.edu</v>
+      </c>
+      <c r="C16" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Ngo Van Phat</v>
+      </c>
+      <c r="B17" t="str">
+        <v>phat@edulms.edu</v>
+      </c>
+      <c r="C17" t="str">
+        <v>teacher</v>
+      </c>
+      <c r="D17" t="str">
+        <v>GV-2002</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Le Van Quyet</v>
+      </c>
+      <c r="B18" t="str">
+        <v>quyet@edulms.edu</v>
+      </c>
+      <c r="C18" t="str">
+        <v>admin</v>
+      </c>
+      <c r="D18" t="str">
+        <v>AD-9001</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Hoang Thi Sen</v>
+      </c>
+      <c r="B19" t="str">
+        <v>sen@edulms.edu</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Học sinh</v>
+      </c>
+      <c r="D19" t="str">
+        <v>HS-9011</v>
+      </c>
+      <c r="E19" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v>invalid_email</v>
+      </c>
+      <c r="C20" t="str">
+        <v>student</v>
+      </c>
+      <c r="D20" t="str">
+        <v>HS-9012</v>
+      </c>
+      <c r="E20" t="str">
+        <v>10A1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Dang Van Tuan</v>
+      </c>
+      <c r="B21" t="str">
+        <v>tuan@edulms.edu</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Giáo viên</v>
+      </c>
+      <c r="D21" t="str">
+        <v>GV-9002</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Mai Thi Uyen</v>
+      </c>
+      <c r="B22" t="str">
+        <v>uyen_invalid</v>
+      </c>
+      <c r="C22" t="str">
+        <v>student</v>
+      </c>
+      <c r="D22" t="str">
+        <v>HS-9013</v>
+      </c>
+      <c r="E22" t="str">
+        <v>12A3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>